<commit_message>
Taktzählung ab 1 wie im DAW: songgen.py --takt-ab, alle Tabellen umgestellt
- tools/struktur.py: shift_bars() verschiebt 'von takt' aller Zeilen
  (Kopie schreiben, zurücklesen, prüfen, dann ersetzen); neue Tabellen
  beginnen bei FIRST_BAR = 1
- tools/songgen.py: --takt-ab N zieht bar:/cues: der show.yaml mit und
  vergleicht den erzeugten Code vorher und nachher
- alle 24 Song-Tabellen, 23 Raster-Kopien und die Vorlage beginnen bei
  Takt 1; der erzeugte Code aller Songs ist unverändert
- Tell It To My Heart: Taktnummern der Blinder in der Show mitgezogen,
  neue Version
- Doku: CLAUDE.md, README, Song-Workflow, Skill new-song

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/songs/Abcdefu_v1/quelle/struktur-raster.xlsx
+++ b/songs/Abcdefu_v1/quelle/struktur-raster.xlsx
@@ -562,7 +562,7 @@
     </row>
     <row r="6" collapsed="1" ht="43.2" customHeight="1">
       <c r="A6" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
@@ -593,7 +593,7 @@
     </row>
     <row r="7" hidden="1" outlineLevel="2">
       <c r="A7" s="4" t="n">
-        <v>0.25</v>
+        <v>1.25</v>
       </c>
       <c r="B7" s="5" t="n"/>
       <c r="C7" s="6" t="n"/>
@@ -605,7 +605,7 @@
     </row>
     <row r="8" hidden="1" outlineLevel="2">
       <c r="A8" s="4" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="B8" s="5" t="n"/>
       <c r="C8" s="6" t="n"/>
@@ -617,7 +617,7 @@
     </row>
     <row r="9" hidden="1" outlineLevel="2">
       <c r="A9" s="4" t="n">
-        <v>0.75</v>
+        <v>1.75</v>
       </c>
       <c r="B9" s="5" t="n"/>
       <c r="C9" s="6" t="n"/>
@@ -629,7 +629,7 @@
     </row>
     <row r="10" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B10" s="5" t="n"/>
       <c r="C10" s="6" t="n"/>
@@ -641,7 +641,7 @@
     </row>
     <row r="11" hidden="1" outlineLevel="2">
       <c r="A11" s="4" t="n">
-        <v>1.25</v>
+        <v>2.25</v>
       </c>
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="6" t="n"/>
@@ -653,7 +653,7 @@
     </row>
     <row r="12" hidden="1" outlineLevel="2">
       <c r="A12" s="4" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="B12" s="5" t="n"/>
       <c r="C12" s="6" t="n"/>
@@ -665,7 +665,7 @@
     </row>
     <row r="13" hidden="1" outlineLevel="2">
       <c r="A13" s="4" t="n">
-        <v>1.75</v>
+        <v>2.75</v>
       </c>
       <c r="B13" s="5" t="n"/>
       <c r="C13" s="6" t="n"/>
@@ -677,7 +677,7 @@
     </row>
     <row r="14" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B14" s="5" t="n"/>
       <c r="C14" s="6" t="n"/>
@@ -689,7 +689,7 @@
     </row>
     <row r="15" hidden="1" outlineLevel="2">
       <c r="A15" s="4" t="n">
-        <v>2.25</v>
+        <v>3.25</v>
       </c>
       <c r="B15" s="5" t="n"/>
       <c r="C15" s="6" t="n"/>
@@ -701,7 +701,7 @@
     </row>
     <row r="16" hidden="1" outlineLevel="2">
       <c r="A16" s="4" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="B16" s="5" t="n"/>
       <c r="C16" s="6" t="n"/>
@@ -713,7 +713,7 @@
     </row>
     <row r="17" hidden="1" outlineLevel="2">
       <c r="A17" s="4" t="n">
-        <v>2.75</v>
+        <v>3.75</v>
       </c>
       <c r="B17" s="5" t="n"/>
       <c r="C17" s="6" t="n"/>
@@ -725,7 +725,7 @@
     </row>
     <row r="18" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A18" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B18" s="5" t="n"/>
       <c r="C18" s="6" t="n"/>
@@ -737,7 +737,7 @@
     </row>
     <row r="19" hidden="1" outlineLevel="2">
       <c r="A19" s="4" t="n">
-        <v>3.25</v>
+        <v>4.25</v>
       </c>
       <c r="B19" s="5" t="n"/>
       <c r="C19" s="6" t="n"/>
@@ -749,7 +749,7 @@
     </row>
     <row r="20" hidden="1" outlineLevel="2">
       <c r="A20" s="4" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="B20" s="5" t="n"/>
       <c r="C20" s="6" t="n"/>
@@ -761,7 +761,7 @@
     </row>
     <row r="21" collapsed="1" ht="43.2" customHeight="1">
       <c r="A21" s="4" t="n">
-        <v>3.75</v>
+        <v>4.75</v>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
@@ -786,7 +786,7 @@
     </row>
     <row r="22" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A22" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B22" s="5" t="n"/>
       <c r="C22" s="12" t="n"/>
@@ -798,7 +798,7 @@
     </row>
     <row r="23" hidden="1" outlineLevel="2">
       <c r="A23" s="4" t="n">
-        <v>4.25</v>
+        <v>5.25</v>
       </c>
       <c r="B23" s="5" t="n"/>
       <c r="C23" s="12" t="n"/>
@@ -810,7 +810,7 @@
     </row>
     <row r="24" hidden="1" outlineLevel="2">
       <c r="A24" s="4" t="n">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
       <c r="B24" s="5" t="n"/>
       <c r="C24" s="12" t="n"/>
@@ -822,7 +822,7 @@
     </row>
     <row r="25" hidden="1" outlineLevel="2">
       <c r="A25" s="4" t="n">
-        <v>4.75</v>
+        <v>5.75</v>
       </c>
       <c r="B25" s="5" t="n"/>
       <c r="C25" s="12" t="n"/>
@@ -834,7 +834,7 @@
     </row>
     <row r="26" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A26" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B26" s="5" t="n"/>
       <c r="C26" s="12" t="n"/>
@@ -846,7 +846,7 @@
     </row>
     <row r="27" hidden="1" outlineLevel="2">
       <c r="A27" s="4" t="n">
-        <v>5.25</v>
+        <v>6.25</v>
       </c>
       <c r="B27" s="5" t="n"/>
       <c r="C27" s="12" t="n"/>
@@ -858,7 +858,7 @@
     </row>
     <row r="28" hidden="1" outlineLevel="2">
       <c r="A28" s="4" t="n">
-        <v>5.5</v>
+        <v>6.5</v>
       </c>
       <c r="B28" s="5" t="n"/>
       <c r="C28" s="12" t="n"/>
@@ -870,7 +870,7 @@
     </row>
     <row r="29" hidden="1" outlineLevel="2">
       <c r="A29" s="4" t="n">
-        <v>5.75</v>
+        <v>6.75</v>
       </c>
       <c r="B29" s="5" t="n"/>
       <c r="C29" s="12" t="n"/>
@@ -882,7 +882,7 @@
     </row>
     <row r="30" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A30" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B30" s="5" t="n"/>
       <c r="C30" s="12" t="n"/>
@@ -894,7 +894,7 @@
     </row>
     <row r="31" hidden="1" outlineLevel="2">
       <c r="A31" s="4" t="n">
-        <v>6.25</v>
+        <v>7.25</v>
       </c>
       <c r="B31" s="5" t="n"/>
       <c r="C31" s="12" t="n"/>
@@ -906,7 +906,7 @@
     </row>
     <row r="32" hidden="1" outlineLevel="2">
       <c r="A32" s="4" t="n">
-        <v>6.5</v>
+        <v>7.5</v>
       </c>
       <c r="B32" s="5" t="n"/>
       <c r="C32" s="12" t="n"/>
@@ -918,7 +918,7 @@
     </row>
     <row r="33" hidden="1" outlineLevel="2">
       <c r="A33" s="4" t="n">
-        <v>6.75</v>
+        <v>7.75</v>
       </c>
       <c r="B33" s="5" t="n"/>
       <c r="C33" s="12" t="n"/>
@@ -930,7 +930,7 @@
     </row>
     <row r="34" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A34" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B34" s="5" t="n"/>
       <c r="C34" s="12" t="n"/>
@@ -942,7 +942,7 @@
     </row>
     <row r="35" hidden="1" outlineLevel="2">
       <c r="A35" s="4" t="n">
-        <v>7.25</v>
+        <v>8.25</v>
       </c>
       <c r="B35" s="5" t="n"/>
       <c r="C35" s="12" t="n"/>
@@ -954,7 +954,7 @@
     </row>
     <row r="36" hidden="1" outlineLevel="2">
       <c r="A36" s="4" t="n">
-        <v>7.5</v>
+        <v>8.5</v>
       </c>
       <c r="B36" s="5" t="n"/>
       <c r="C36" s="12" t="n"/>
@@ -966,7 +966,7 @@
     </row>
     <row r="37" hidden="1" outlineLevel="2">
       <c r="A37" s="4" t="n">
-        <v>7.75</v>
+        <v>8.75</v>
       </c>
       <c r="B37" s="5" t="n"/>
       <c r="C37" s="12" t="n"/>
@@ -978,7 +978,7 @@
     </row>
     <row r="38" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A38" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B38" s="5" t="n"/>
       <c r="C38" s="12" t="n"/>
@@ -990,7 +990,7 @@
     </row>
     <row r="39" hidden="1" outlineLevel="2">
       <c r="A39" s="4" t="n">
-        <v>8.25</v>
+        <v>9.25</v>
       </c>
       <c r="B39" s="5" t="n"/>
       <c r="C39" s="12" t="n"/>
@@ -1002,7 +1002,7 @@
     </row>
     <row r="40" hidden="1" outlineLevel="2">
       <c r="A40" s="4" t="n">
-        <v>8.5</v>
+        <v>9.5</v>
       </c>
       <c r="B40" s="5" t="n"/>
       <c r="C40" s="12" t="n"/>
@@ -1014,7 +1014,7 @@
     </row>
     <row r="41" hidden="1" outlineLevel="2">
       <c r="A41" s="4" t="n">
-        <v>8.75</v>
+        <v>9.75</v>
       </c>
       <c r="B41" s="5" t="n"/>
       <c r="C41" s="12" t="n"/>
@@ -1026,7 +1026,7 @@
     </row>
     <row r="42" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A42" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B42" s="5" t="n"/>
       <c r="C42" s="12" t="n"/>
@@ -1038,7 +1038,7 @@
     </row>
     <row r="43" hidden="1" outlineLevel="2">
       <c r="A43" s="4" t="n">
-        <v>9.25</v>
+        <v>10.25</v>
       </c>
       <c r="B43" s="5" t="n"/>
       <c r="C43" s="12" t="n"/>
@@ -1050,7 +1050,7 @@
     </row>
     <row r="44" hidden="1" outlineLevel="2">
       <c r="A44" s="4" t="n">
-        <v>9.5</v>
+        <v>10.5</v>
       </c>
       <c r="B44" s="5" t="n"/>
       <c r="C44" s="12" t="n"/>
@@ -1062,7 +1062,7 @@
     </row>
     <row r="45" hidden="1" outlineLevel="2">
       <c r="A45" s="4" t="n">
-        <v>9.75</v>
+        <v>10.75</v>
       </c>
       <c r="B45" s="5" t="n"/>
       <c r="C45" s="12" t="n"/>
@@ -1074,7 +1074,7 @@
     </row>
     <row r="46" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A46" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B46" s="5" t="n"/>
       <c r="C46" s="12" t="n"/>
@@ -1086,7 +1086,7 @@
     </row>
     <row r="47" hidden="1" outlineLevel="2">
       <c r="A47" s="4" t="n">
-        <v>10.25</v>
+        <v>11.25</v>
       </c>
       <c r="B47" s="5" t="n"/>
       <c r="C47" s="12" t="n"/>
@@ -1098,7 +1098,7 @@
     </row>
     <row r="48" hidden="1" outlineLevel="2">
       <c r="A48" s="4" t="n">
-        <v>10.5</v>
+        <v>11.5</v>
       </c>
       <c r="B48" s="5" t="n"/>
       <c r="C48" s="12" t="n"/>
@@ -1110,7 +1110,7 @@
     </row>
     <row r="49" hidden="1" outlineLevel="2">
       <c r="A49" s="4" t="n">
-        <v>10.75</v>
+        <v>11.75</v>
       </c>
       <c r="B49" s="5" t="n"/>
       <c r="C49" s="12" t="n"/>
@@ -1122,7 +1122,7 @@
     </row>
     <row r="50" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A50" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B50" s="5" t="n"/>
       <c r="C50" s="12" t="n"/>
@@ -1134,7 +1134,7 @@
     </row>
     <row r="51" hidden="1" outlineLevel="2">
       <c r="A51" s="4" t="n">
-        <v>11.25</v>
+        <v>12.25</v>
       </c>
       <c r="B51" s="5" t="n"/>
       <c r="C51" s="12" t="n"/>
@@ -1146,7 +1146,7 @@
     </row>
     <row r="52" collapsed="1" ht="28.8" customHeight="1">
       <c r="A52" s="4" t="n">
-        <v>11.5</v>
+        <v>12.5</v>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
@@ -1176,7 +1176,7 @@
     </row>
     <row r="53" hidden="1" outlineLevel="2">
       <c r="A53" s="4" t="n">
-        <v>11.75</v>
+        <v>12.75</v>
       </c>
       <c r="B53" s="5" t="n"/>
       <c r="C53" s="6" t="n"/>
@@ -1188,7 +1188,7 @@
     </row>
     <row r="54" collapsed="1" ht="28.8" customHeight="1">
       <c r="A54" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
@@ -1218,7 +1218,7 @@
     </row>
     <row r="55" hidden="1" outlineLevel="2">
       <c r="A55" s="4" t="n">
-        <v>12.25</v>
+        <v>13.25</v>
       </c>
       <c r="B55" s="5" t="n"/>
       <c r="C55" s="6" t="n"/>
@@ -1230,7 +1230,7 @@
     </row>
     <row r="56" hidden="1" outlineLevel="2">
       <c r="A56" s="4" t="n">
-        <v>12.5</v>
+        <v>13.5</v>
       </c>
       <c r="B56" s="5" t="n"/>
       <c r="C56" s="6" t="n"/>
@@ -1242,7 +1242,7 @@
     </row>
     <row r="57" hidden="1" outlineLevel="2">
       <c r="A57" s="4" t="n">
-        <v>12.75</v>
+        <v>13.75</v>
       </c>
       <c r="B57" s="5" t="n"/>
       <c r="C57" s="6" t="n"/>
@@ -1254,7 +1254,7 @@
     </row>
     <row r="58" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A58" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B58" s="5" t="n"/>
       <c r="C58" s="6" t="n"/>
@@ -1266,7 +1266,7 @@
     </row>
     <row r="59" hidden="1" outlineLevel="2">
       <c r="A59" s="4" t="n">
-        <v>13.25</v>
+        <v>14.25</v>
       </c>
       <c r="B59" s="5" t="n"/>
       <c r="C59" s="6" t="n"/>
@@ -1278,7 +1278,7 @@
     </row>
     <row r="60" hidden="1" outlineLevel="2">
       <c r="A60" s="4" t="n">
-        <v>13.5</v>
+        <v>14.5</v>
       </c>
       <c r="B60" s="5" t="n"/>
       <c r="C60" s="6" t="n"/>
@@ -1290,7 +1290,7 @@
     </row>
     <row r="61" hidden="1" outlineLevel="2">
       <c r="A61" s="4" t="n">
-        <v>13.75</v>
+        <v>14.75</v>
       </c>
       <c r="B61" s="5" t="n"/>
       <c r="C61" s="6" t="n"/>
@@ -1302,7 +1302,7 @@
     </row>
     <row r="62" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A62" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B62" s="5" t="n"/>
       <c r="C62" s="6" t="n"/>
@@ -1314,7 +1314,7 @@
     </row>
     <row r="63" hidden="1" outlineLevel="2">
       <c r="A63" s="4" t="n">
-        <v>14.25</v>
+        <v>15.25</v>
       </c>
       <c r="B63" s="5" t="n"/>
       <c r="C63" s="6" t="n"/>
@@ -1326,7 +1326,7 @@
     </row>
     <row r="64" hidden="1" outlineLevel="2">
       <c r="A64" s="4" t="n">
-        <v>14.5</v>
+        <v>15.5</v>
       </c>
       <c r="B64" s="5" t="n"/>
       <c r="C64" s="6" t="n"/>
@@ -1338,7 +1338,7 @@
     </row>
     <row r="65" hidden="1" outlineLevel="2">
       <c r="A65" s="4" t="n">
-        <v>14.75</v>
+        <v>15.75</v>
       </c>
       <c r="B65" s="5" t="n"/>
       <c r="C65" s="6" t="n"/>
@@ -1350,7 +1350,7 @@
     </row>
     <row r="66" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A66" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B66" s="5" t="n"/>
       <c r="C66" s="6" t="n"/>
@@ -1362,7 +1362,7 @@
     </row>
     <row r="67" hidden="1" outlineLevel="2">
       <c r="A67" s="4" t="n">
-        <v>15.25</v>
+        <v>16.25</v>
       </c>
       <c r="B67" s="5" t="n"/>
       <c r="C67" s="6" t="n"/>
@@ -1374,7 +1374,7 @@
     </row>
     <row r="68" hidden="1" outlineLevel="2">
       <c r="A68" s="4" t="n">
-        <v>15.5</v>
+        <v>16.5</v>
       </c>
       <c r="B68" s="5" t="n"/>
       <c r="C68" s="6" t="n"/>
@@ -1386,7 +1386,7 @@
     </row>
     <row r="69" hidden="1" outlineLevel="2">
       <c r="A69" s="4" t="n">
-        <v>15.75</v>
+        <v>16.75</v>
       </c>
       <c r="B69" s="5" t="n"/>
       <c r="C69" s="6" t="n"/>
@@ -1398,7 +1398,7 @@
     </row>
     <row r="70" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A70" s="4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B70" s="5" t="n"/>
       <c r="C70" s="6" t="n"/>
@@ -1410,7 +1410,7 @@
     </row>
     <row r="71" hidden="1" outlineLevel="2">
       <c r="A71" s="4" t="n">
-        <v>16.25</v>
+        <v>17.25</v>
       </c>
       <c r="B71" s="5" t="n"/>
       <c r="C71" s="6" t="n"/>
@@ -1422,7 +1422,7 @@
     </row>
     <row r="72" hidden="1" outlineLevel="2">
       <c r="A72" s="4" t="n">
-        <v>16.5</v>
+        <v>17.5</v>
       </c>
       <c r="B72" s="5" t="n"/>
       <c r="C72" s="6" t="n"/>
@@ -1434,7 +1434,7 @@
     </row>
     <row r="73" hidden="1" outlineLevel="2">
       <c r="A73" s="4" t="n">
-        <v>16.75</v>
+        <v>17.75</v>
       </c>
       <c r="B73" s="5" t="n"/>
       <c r="C73" s="6" t="n"/>
@@ -1446,7 +1446,7 @@
     </row>
     <row r="74" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A74" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B74" s="5" t="n"/>
       <c r="C74" s="6" t="n"/>
@@ -1458,7 +1458,7 @@
     </row>
     <row r="75" hidden="1" outlineLevel="2">
       <c r="A75" s="4" t="n">
-        <v>17.25</v>
+        <v>18.25</v>
       </c>
       <c r="B75" s="5" t="n"/>
       <c r="C75" s="6" t="n"/>
@@ -1470,7 +1470,7 @@
     </row>
     <row r="76" hidden="1" outlineLevel="2">
       <c r="A76" s="4" t="n">
-        <v>17.5</v>
+        <v>18.5</v>
       </c>
       <c r="B76" s="5" t="n"/>
       <c r="C76" s="6" t="n"/>
@@ -1482,7 +1482,7 @@
     </row>
     <row r="77" hidden="1" outlineLevel="2">
       <c r="A77" s="4" t="n">
-        <v>17.75</v>
+        <v>18.75</v>
       </c>
       <c r="B77" s="5" t="n"/>
       <c r="C77" s="6" t="n"/>
@@ -1494,7 +1494,7 @@
     </row>
     <row r="78" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A78" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B78" s="5" t="n"/>
       <c r="C78" s="6" t="n"/>
@@ -1506,7 +1506,7 @@
     </row>
     <row r="79" hidden="1" outlineLevel="2">
       <c r="A79" s="4" t="n">
-        <v>18.25</v>
+        <v>19.25</v>
       </c>
       <c r="B79" s="5" t="n"/>
       <c r="C79" s="6" t="n"/>
@@ -1518,7 +1518,7 @@
     </row>
     <row r="80" hidden="1" outlineLevel="2">
       <c r="A80" s="4" t="n">
-        <v>18.5</v>
+        <v>19.5</v>
       </c>
       <c r="B80" s="5" t="n"/>
       <c r="C80" s="6" t="n"/>
@@ -1530,7 +1530,7 @@
     </row>
     <row r="81" hidden="1" outlineLevel="2">
       <c r="A81" s="4" t="n">
-        <v>18.75</v>
+        <v>19.75</v>
       </c>
       <c r="B81" s="5" t="n"/>
       <c r="C81" s="6" t="n"/>
@@ -1542,7 +1542,7 @@
     </row>
     <row r="82" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A82" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B82" s="5" t="n"/>
       <c r="C82" s="6" t="n"/>
@@ -1554,7 +1554,7 @@
     </row>
     <row r="83" hidden="1" outlineLevel="2">
       <c r="A83" s="4" t="n">
-        <v>19.25</v>
+        <v>20.25</v>
       </c>
       <c r="B83" s="5" t="n"/>
       <c r="C83" s="6" t="n"/>
@@ -1566,7 +1566,7 @@
     </row>
     <row r="84" hidden="1" outlineLevel="2">
       <c r="A84" s="4" t="n">
-        <v>19.5</v>
+        <v>20.5</v>
       </c>
       <c r="B84" s="5" t="n"/>
       <c r="C84" s="6" t="n"/>
@@ -1578,7 +1578,7 @@
     </row>
     <row r="85" hidden="1" outlineLevel="2">
       <c r="A85" s="4" t="n">
-        <v>19.75</v>
+        <v>20.75</v>
       </c>
       <c r="B85" s="5" t="n"/>
       <c r="C85" s="6" t="n"/>
@@ -1590,7 +1590,7 @@
     </row>
     <row r="86" collapsed="1" ht="28.8" customHeight="1">
       <c r="A86" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
@@ -1620,7 +1620,7 @@
     </row>
     <row r="87" hidden="1" outlineLevel="2">
       <c r="A87" s="4" t="n">
-        <v>20.25</v>
+        <v>21.25</v>
       </c>
       <c r="B87" s="5" t="n"/>
       <c r="C87" s="6" t="n"/>
@@ -1632,7 +1632,7 @@
     </row>
     <row r="88" hidden="1" outlineLevel="2">
       <c r="A88" s="4" t="n">
-        <v>20.5</v>
+        <v>21.5</v>
       </c>
       <c r="B88" s="5" t="n"/>
       <c r="C88" s="6" t="n"/>
@@ -1644,7 +1644,7 @@
     </row>
     <row r="89" hidden="1" outlineLevel="2">
       <c r="A89" s="4" t="n">
-        <v>20.75</v>
+        <v>21.75</v>
       </c>
       <c r="B89" s="5" t="n"/>
       <c r="C89" s="6" t="n"/>
@@ -1656,7 +1656,7 @@
     </row>
     <row r="90" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A90" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B90" s="5" t="n"/>
       <c r="C90" s="6" t="n"/>
@@ -1668,7 +1668,7 @@
     </row>
     <row r="91" hidden="1" outlineLevel="2">
       <c r="A91" s="4" t="n">
-        <v>21.25</v>
+        <v>22.25</v>
       </c>
       <c r="B91" s="5" t="n"/>
       <c r="C91" s="6" t="n"/>
@@ -1680,7 +1680,7 @@
     </row>
     <row r="92" hidden="1" outlineLevel="2">
       <c r="A92" s="4" t="n">
-        <v>21.5</v>
+        <v>22.5</v>
       </c>
       <c r="B92" s="5" t="n"/>
       <c r="C92" s="6" t="n"/>
@@ -1692,7 +1692,7 @@
     </row>
     <row r="93" hidden="1" outlineLevel="2">
       <c r="A93" s="4" t="n">
-        <v>21.75</v>
+        <v>22.75</v>
       </c>
       <c r="B93" s="5" t="n"/>
       <c r="C93" s="6" t="n"/>
@@ -1704,7 +1704,7 @@
     </row>
     <row r="94" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A94" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B94" s="5" t="n"/>
       <c r="C94" s="6" t="n"/>
@@ -1716,7 +1716,7 @@
     </row>
     <row r="95" hidden="1" outlineLevel="2">
       <c r="A95" s="4" t="n">
-        <v>22.25</v>
+        <v>23.25</v>
       </c>
       <c r="B95" s="5" t="n"/>
       <c r="C95" s="6" t="n"/>
@@ -1728,7 +1728,7 @@
     </row>
     <row r="96" hidden="1" outlineLevel="2">
       <c r="A96" s="4" t="n">
-        <v>22.5</v>
+        <v>23.5</v>
       </c>
       <c r="B96" s="5" t="n"/>
       <c r="C96" s="6" t="n"/>
@@ -1740,7 +1740,7 @@
     </row>
     <row r="97" hidden="1" outlineLevel="2">
       <c r="A97" s="4" t="n">
-        <v>22.75</v>
+        <v>23.75</v>
       </c>
       <c r="B97" s="5" t="n"/>
       <c r="C97" s="6" t="n"/>
@@ -1752,7 +1752,7 @@
     </row>
     <row r="98" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A98" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B98" s="5" t="n"/>
       <c r="C98" s="6" t="n"/>
@@ -1764,7 +1764,7 @@
     </row>
     <row r="99" hidden="1" outlineLevel="2">
       <c r="A99" s="4" t="n">
-        <v>23.25</v>
+        <v>24.25</v>
       </c>
       <c r="B99" s="5" t="n"/>
       <c r="C99" s="6" t="n"/>
@@ -1776,7 +1776,7 @@
     </row>
     <row r="100" hidden="1" outlineLevel="2">
       <c r="A100" s="4" t="n">
-        <v>23.5</v>
+        <v>24.5</v>
       </c>
       <c r="B100" s="5" t="n"/>
       <c r="C100" s="6" t="n"/>
@@ -1788,7 +1788,7 @@
     </row>
     <row r="101" hidden="1" outlineLevel="2">
       <c r="A101" s="4" t="n">
-        <v>23.75</v>
+        <v>24.75</v>
       </c>
       <c r="B101" s="5" t="n"/>
       <c r="C101" s="6" t="n"/>
@@ -1800,7 +1800,7 @@
     </row>
     <row r="102" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A102" s="4" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B102" s="5" t="n"/>
       <c r="C102" s="6" t="n"/>
@@ -1812,7 +1812,7 @@
     </row>
     <row r="103" hidden="1" outlineLevel="2">
       <c r="A103" s="4" t="n">
-        <v>24.25</v>
+        <v>25.25</v>
       </c>
       <c r="B103" s="5" t="n"/>
       <c r="C103" s="6" t="n"/>
@@ -1824,7 +1824,7 @@
     </row>
     <row r="104" hidden="1" outlineLevel="2">
       <c r="A104" s="4" t="n">
-        <v>24.5</v>
+        <v>25.5</v>
       </c>
       <c r="B104" s="5" t="n"/>
       <c r="C104" s="6" t="n"/>
@@ -1836,7 +1836,7 @@
     </row>
     <row r="105" hidden="1" outlineLevel="2">
       <c r="A105" s="4" t="n">
-        <v>24.75</v>
+        <v>25.75</v>
       </c>
       <c r="B105" s="5" t="n"/>
       <c r="C105" s="6" t="n"/>
@@ -1848,7 +1848,7 @@
     </row>
     <row r="106" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A106" s="4" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B106" s="5" t="n"/>
       <c r="C106" s="6" t="n"/>
@@ -1860,7 +1860,7 @@
     </row>
     <row r="107" hidden="1" outlineLevel="2">
       <c r="A107" s="4" t="n">
-        <v>25.25</v>
+        <v>26.25</v>
       </c>
       <c r="B107" s="5" t="n"/>
       <c r="C107" s="6" t="n"/>
@@ -1872,7 +1872,7 @@
     </row>
     <row r="108" hidden="1" outlineLevel="2">
       <c r="A108" s="4" t="n">
-        <v>25.5</v>
+        <v>26.5</v>
       </c>
       <c r="B108" s="5" t="n"/>
       <c r="C108" s="6" t="n"/>
@@ -1884,7 +1884,7 @@
     </row>
     <row r="109" hidden="1" outlineLevel="2">
       <c r="A109" s="4" t="n">
-        <v>25.75</v>
+        <v>26.75</v>
       </c>
       <c r="B109" s="5" t="n"/>
       <c r="C109" s="6" t="n"/>
@@ -1896,7 +1896,7 @@
     </row>
     <row r="110" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A110" s="4" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B110" s="5" t="n"/>
       <c r="C110" s="6" t="n"/>
@@ -1908,7 +1908,7 @@
     </row>
     <row r="111" hidden="1" outlineLevel="2">
       <c r="A111" s="4" t="n">
-        <v>26.25</v>
+        <v>27.25</v>
       </c>
       <c r="B111" s="5" t="n"/>
       <c r="C111" s="6" t="n"/>
@@ -1920,7 +1920,7 @@
     </row>
     <row r="112" hidden="1" outlineLevel="2">
       <c r="A112" s="4" t="n">
-        <v>26.5</v>
+        <v>27.5</v>
       </c>
       <c r="B112" s="5" t="n"/>
       <c r="C112" s="6" t="n"/>
@@ -1932,7 +1932,7 @@
     </row>
     <row r="113" hidden="1" outlineLevel="2">
       <c r="A113" s="4" t="n">
-        <v>26.75</v>
+        <v>27.75</v>
       </c>
       <c r="B113" s="5" t="n"/>
       <c r="C113" s="6" t="n"/>
@@ -1944,7 +1944,7 @@
     </row>
     <row r="114" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A114" s="4" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B114" s="5" t="n"/>
       <c r="C114" s="6" t="n"/>
@@ -1956,7 +1956,7 @@
     </row>
     <row r="115" hidden="1" outlineLevel="2">
       <c r="A115" s="4" t="n">
-        <v>27.25</v>
+        <v>28.25</v>
       </c>
       <c r="B115" s="5" t="n"/>
       <c r="C115" s="6" t="n"/>
@@ -1968,7 +1968,7 @@
     </row>
     <row r="116" hidden="1" outlineLevel="2">
       <c r="A116" s="4" t="n">
-        <v>27.5</v>
+        <v>28.5</v>
       </c>
       <c r="B116" s="5" t="n"/>
       <c r="C116" s="6" t="n"/>
@@ -1980,7 +1980,7 @@
     </row>
     <row r="117" hidden="1" outlineLevel="2">
       <c r="A117" s="4" t="n">
-        <v>27.75</v>
+        <v>28.75</v>
       </c>
       <c r="B117" s="5" t="n"/>
       <c r="C117" s="6" t="n"/>
@@ -1992,7 +1992,7 @@
     </row>
     <row r="118" collapsed="1" ht="86.40000000000001" customHeight="1">
       <c r="A118" s="4" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B118" s="5" t="inlineStr">
         <is>
@@ -2024,7 +2024,7 @@
     </row>
     <row r="119" hidden="1" outlineLevel="2">
       <c r="A119" s="4" t="n">
-        <v>28.25</v>
+        <v>29.25</v>
       </c>
       <c r="B119" s="5" t="n"/>
       <c r="C119" s="6" t="n"/>
@@ -2036,7 +2036,7 @@
     </row>
     <row r="120" hidden="1" outlineLevel="2">
       <c r="A120" s="4" t="n">
-        <v>28.5</v>
+        <v>29.5</v>
       </c>
       <c r="B120" s="5" t="n"/>
       <c r="C120" s="6" t="n"/>
@@ -2048,7 +2048,7 @@
     </row>
     <row r="121" hidden="1" outlineLevel="2">
       <c r="A121" s="4" t="n">
-        <v>28.75</v>
+        <v>29.75</v>
       </c>
       <c r="B121" s="5" t="n"/>
       <c r="C121" s="6" t="n"/>
@@ -2060,7 +2060,7 @@
     </row>
     <row r="122" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A122" s="4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B122" s="5" t="n"/>
       <c r="C122" s="6" t="n"/>
@@ -2072,7 +2072,7 @@
     </row>
     <row r="123" hidden="1" outlineLevel="2">
       <c r="A123" s="4" t="n">
-        <v>29.25</v>
+        <v>30.25</v>
       </c>
       <c r="B123" s="5" t="n"/>
       <c r="C123" s="6" t="n"/>
@@ -2084,7 +2084,7 @@
     </row>
     <row r="124" hidden="1" outlineLevel="2">
       <c r="A124" s="4" t="n">
-        <v>29.5</v>
+        <v>30.5</v>
       </c>
       <c r="B124" s="5" t="n"/>
       <c r="C124" s="6" t="n"/>
@@ -2096,7 +2096,7 @@
     </row>
     <row r="125" hidden="1" outlineLevel="2">
       <c r="A125" s="4" t="n">
-        <v>29.75</v>
+        <v>30.75</v>
       </c>
       <c r="B125" s="5" t="n"/>
       <c r="C125" s="6" t="n"/>
@@ -2108,7 +2108,7 @@
     </row>
     <row r="126" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A126" s="4" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B126" s="5" t="n"/>
       <c r="C126" s="6" t="n"/>
@@ -2120,7 +2120,7 @@
     </row>
     <row r="127" hidden="1" outlineLevel="2">
       <c r="A127" s="4" t="n">
-        <v>30.25</v>
+        <v>31.25</v>
       </c>
       <c r="B127" s="5" t="n"/>
       <c r="C127" s="6" t="n"/>
@@ -2132,7 +2132,7 @@
     </row>
     <row r="128" hidden="1" outlineLevel="2">
       <c r="A128" s="4" t="n">
-        <v>30.5</v>
+        <v>31.5</v>
       </c>
       <c r="B128" s="5" t="n"/>
       <c r="C128" s="6" t="n"/>
@@ -2144,7 +2144,7 @@
     </row>
     <row r="129" hidden="1" outlineLevel="2">
       <c r="A129" s="4" t="n">
-        <v>30.75</v>
+        <v>31.75</v>
       </c>
       <c r="B129" s="5" t="n"/>
       <c r="C129" s="6" t="n"/>
@@ -2156,7 +2156,7 @@
     </row>
     <row r="130" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A130" s="4" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B130" s="5" t="n"/>
       <c r="C130" s="6" t="n"/>
@@ -2168,7 +2168,7 @@
     </row>
     <row r="131" hidden="1" outlineLevel="2">
       <c r="A131" s="4" t="n">
-        <v>31.25</v>
+        <v>32.25</v>
       </c>
       <c r="B131" s="5" t="n"/>
       <c r="C131" s="6" t="n"/>
@@ -2180,7 +2180,7 @@
     </row>
     <row r="132" hidden="1" outlineLevel="2">
       <c r="A132" s="4" t="n">
-        <v>31.5</v>
+        <v>32.5</v>
       </c>
       <c r="B132" s="5" t="n"/>
       <c r="C132" s="6" t="n"/>
@@ -2192,7 +2192,7 @@
     </row>
     <row r="133" hidden="1" outlineLevel="2">
       <c r="A133" s="4" t="n">
-        <v>31.75</v>
+        <v>32.75</v>
       </c>
       <c r="B133" s="5" t="n"/>
       <c r="C133" s="6" t="n"/>
@@ -2204,7 +2204,7 @@
     </row>
     <row r="134" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A134" s="4" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B134" s="5" t="n"/>
       <c r="C134" s="6" t="n"/>
@@ -2216,7 +2216,7 @@
     </row>
     <row r="135" hidden="1" outlineLevel="2">
       <c r="A135" s="4" t="n">
-        <v>32.25</v>
+        <v>33.25</v>
       </c>
       <c r="B135" s="5" t="n"/>
       <c r="C135" s="6" t="n"/>
@@ -2228,7 +2228,7 @@
     </row>
     <row r="136" hidden="1" outlineLevel="2">
       <c r="A136" s="4" t="n">
-        <v>32.5</v>
+        <v>33.5</v>
       </c>
       <c r="B136" s="5" t="n"/>
       <c r="C136" s="6" t="n"/>
@@ -2240,7 +2240,7 @@
     </row>
     <row r="137" hidden="1" outlineLevel="2">
       <c r="A137" s="4" t="n">
-        <v>32.75</v>
+        <v>33.75</v>
       </c>
       <c r="B137" s="5" t="n"/>
       <c r="C137" s="6" t="n"/>
@@ -2252,7 +2252,7 @@
     </row>
     <row r="138" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A138" s="4" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B138" s="5" t="n"/>
       <c r="C138" s="6" t="n"/>
@@ -2264,7 +2264,7 @@
     </row>
     <row r="139" hidden="1" outlineLevel="2">
       <c r="A139" s="4" t="n">
-        <v>33.25</v>
+        <v>34.25</v>
       </c>
       <c r="B139" s="5" t="n"/>
       <c r="C139" s="6" t="n"/>
@@ -2276,7 +2276,7 @@
     </row>
     <row r="140" hidden="1" outlineLevel="2">
       <c r="A140" s="4" t="n">
-        <v>33.5</v>
+        <v>34.5</v>
       </c>
       <c r="B140" s="5" t="n"/>
       <c r="C140" s="6" t="n"/>
@@ -2288,7 +2288,7 @@
     </row>
     <row r="141" hidden="1" outlineLevel="2">
       <c r="A141" s="4" t="n">
-        <v>33.75</v>
+        <v>34.75</v>
       </c>
       <c r="B141" s="5" t="n"/>
       <c r="C141" s="6" t="n"/>
@@ -2300,7 +2300,7 @@
     </row>
     <row r="142" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A142" s="4" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B142" s="5" t="n"/>
       <c r="C142" s="6" t="n"/>
@@ -2312,7 +2312,7 @@
     </row>
     <row r="143" hidden="1" outlineLevel="2">
       <c r="A143" s="4" t="n">
-        <v>34.25</v>
+        <v>35.25</v>
       </c>
       <c r="B143" s="5" t="n"/>
       <c r="C143" s="6" t="n"/>
@@ -2324,7 +2324,7 @@
     </row>
     <row r="144" hidden="1" outlineLevel="2">
       <c r="A144" s="4" t="n">
-        <v>34.5</v>
+        <v>35.5</v>
       </c>
       <c r="B144" s="5" t="n"/>
       <c r="C144" s="6" t="n"/>
@@ -2336,7 +2336,7 @@
     </row>
     <row r="145" hidden="1" outlineLevel="2">
       <c r="A145" s="4" t="n">
-        <v>34.75</v>
+        <v>35.75</v>
       </c>
       <c r="B145" s="5" t="n"/>
       <c r="C145" s="6" t="n"/>
@@ -2348,7 +2348,7 @@
     </row>
     <row r="146" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A146" s="4" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B146" s="5" t="n"/>
       <c r="C146" s="6" t="n"/>
@@ -2360,7 +2360,7 @@
     </row>
     <row r="147" hidden="1" outlineLevel="2">
       <c r="A147" s="4" t="n">
-        <v>35.25</v>
+        <v>36.25</v>
       </c>
       <c r="B147" s="5" t="n"/>
       <c r="C147" s="6" t="n"/>
@@ -2372,7 +2372,7 @@
     </row>
     <row r="148" hidden="1" outlineLevel="2">
       <c r="A148" s="4" t="n">
-        <v>35.5</v>
+        <v>36.5</v>
       </c>
       <c r="B148" s="5" t="n"/>
       <c r="C148" s="6" t="n"/>
@@ -2384,7 +2384,7 @@
     </row>
     <row r="149" hidden="1" outlineLevel="2">
       <c r="A149" s="4" t="n">
-        <v>35.75</v>
+        <v>36.75</v>
       </c>
       <c r="B149" s="5" t="n"/>
       <c r="C149" s="6" t="n"/>
@@ -2396,7 +2396,7 @@
     </row>
     <row r="150" collapsed="1" ht="28.8" customHeight="1">
       <c r="A150" s="4" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B150" s="5" t="inlineStr">
         <is>
@@ -2428,7 +2428,7 @@
     </row>
     <row r="151" hidden="1" outlineLevel="2">
       <c r="A151" s="4" t="n">
-        <v>36.25</v>
+        <v>37.25</v>
       </c>
       <c r="B151" s="5" t="n"/>
       <c r="C151" s="6" t="n"/>
@@ -2440,7 +2440,7 @@
     </row>
     <row r="152" hidden="1" outlineLevel="2">
       <c r="A152" s="4" t="n">
-        <v>36.5</v>
+        <v>37.5</v>
       </c>
       <c r="B152" s="5" t="n"/>
       <c r="C152" s="6" t="n"/>
@@ -2452,7 +2452,7 @@
     </row>
     <row r="153" hidden="1" outlineLevel="2">
       <c r="A153" s="4" t="n">
-        <v>36.75</v>
+        <v>37.75</v>
       </c>
       <c r="B153" s="5" t="n"/>
       <c r="C153" s="6" t="n"/>
@@ -2464,7 +2464,7 @@
     </row>
     <row r="154" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A154" s="4" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B154" s="5" t="n"/>
       <c r="C154" s="6" t="n"/>
@@ -2476,7 +2476,7 @@
     </row>
     <row r="155" hidden="1" outlineLevel="2">
       <c r="A155" s="4" t="n">
-        <v>37.25</v>
+        <v>38.25</v>
       </c>
       <c r="B155" s="5" t="n"/>
       <c r="C155" s="6" t="n"/>
@@ -2488,7 +2488,7 @@
     </row>
     <row r="156" hidden="1" outlineLevel="2">
       <c r="A156" s="4" t="n">
-        <v>37.5</v>
+        <v>38.5</v>
       </c>
       <c r="B156" s="5" t="n"/>
       <c r="C156" s="6" t="n"/>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="157" hidden="1" outlineLevel="2">
       <c r="A157" s="4" t="n">
-        <v>37.75</v>
+        <v>38.75</v>
       </c>
       <c r="B157" s="5" t="n"/>
       <c r="C157" s="6" t="n"/>
@@ -2512,7 +2512,7 @@
     </row>
     <row r="158" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A158" s="4" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B158" s="5" t="n"/>
       <c r="C158" s="6" t="n"/>
@@ -2524,7 +2524,7 @@
     </row>
     <row r="159" hidden="1" outlineLevel="2">
       <c r="A159" s="4" t="n">
-        <v>38.25</v>
+        <v>39.25</v>
       </c>
       <c r="B159" s="5" t="n"/>
       <c r="C159" s="6" t="n"/>
@@ -2536,7 +2536,7 @@
     </row>
     <row r="160" hidden="1" outlineLevel="2">
       <c r="A160" s="4" t="n">
-        <v>38.5</v>
+        <v>39.5</v>
       </c>
       <c r="B160" s="5" t="n"/>
       <c r="C160" s="6" t="n"/>
@@ -2548,7 +2548,7 @@
     </row>
     <row r="161" hidden="1" outlineLevel="2">
       <c r="A161" s="4" t="n">
-        <v>38.75</v>
+        <v>39.75</v>
       </c>
       <c r="B161" s="5" t="n"/>
       <c r="C161" s="6" t="n"/>
@@ -2560,7 +2560,7 @@
     </row>
     <row r="162" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A162" s="4" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B162" s="5" t="n"/>
       <c r="C162" s="6" t="n"/>
@@ -2572,7 +2572,7 @@
     </row>
     <row r="163" hidden="1" outlineLevel="2">
       <c r="A163" s="4" t="n">
-        <v>39.25</v>
+        <v>40.25</v>
       </c>
       <c r="B163" s="5" t="n"/>
       <c r="C163" s="6" t="n"/>
@@ -2584,7 +2584,7 @@
     </row>
     <row r="164" hidden="1" outlineLevel="2">
       <c r="A164" s="4" t="n">
-        <v>39.5</v>
+        <v>40.5</v>
       </c>
       <c r="B164" s="5" t="n"/>
       <c r="C164" s="6" t="n"/>
@@ -2596,7 +2596,7 @@
     </row>
     <row r="165" hidden="1" outlineLevel="2">
       <c r="A165" s="4" t="n">
-        <v>39.75</v>
+        <v>40.75</v>
       </c>
       <c r="B165" s="5" t="n"/>
       <c r="C165" s="6" t="n"/>
@@ -2608,7 +2608,7 @@
     </row>
     <row r="166" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A166" s="4" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B166" s="5" t="n"/>
       <c r="C166" s="6" t="n"/>
@@ -2620,7 +2620,7 @@
     </row>
     <row r="167" hidden="1" outlineLevel="2">
       <c r="A167" s="4" t="n">
-        <v>40.25</v>
+        <v>41.25</v>
       </c>
       <c r="B167" s="5" t="n"/>
       <c r="C167" s="6" t="n"/>
@@ -2632,7 +2632,7 @@
     </row>
     <row r="168" hidden="1" outlineLevel="2">
       <c r="A168" s="4" t="n">
-        <v>40.5</v>
+        <v>41.5</v>
       </c>
       <c r="B168" s="5" t="n"/>
       <c r="C168" s="6" t="n"/>
@@ -2644,7 +2644,7 @@
     </row>
     <row r="169" hidden="1" outlineLevel="2">
       <c r="A169" s="4" t="n">
-        <v>40.75</v>
+        <v>41.75</v>
       </c>
       <c r="B169" s="5" t="n"/>
       <c r="C169" s="6" t="n"/>
@@ -2656,7 +2656,7 @@
     </row>
     <row r="170" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A170" s="4" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B170" s="5" t="n"/>
       <c r="C170" s="6" t="n"/>
@@ -2668,7 +2668,7 @@
     </row>
     <row r="171" hidden="1" outlineLevel="2">
       <c r="A171" s="4" t="n">
-        <v>41.25</v>
+        <v>42.25</v>
       </c>
       <c r="B171" s="5" t="n"/>
       <c r="C171" s="6" t="n"/>
@@ -2680,7 +2680,7 @@
     </row>
     <row r="172" hidden="1" outlineLevel="2">
       <c r="A172" s="4" t="n">
-        <v>41.5</v>
+        <v>42.5</v>
       </c>
       <c r="B172" s="5" t="n"/>
       <c r="C172" s="6" t="n"/>
@@ -2692,7 +2692,7 @@
     </row>
     <row r="173" hidden="1" outlineLevel="2">
       <c r="A173" s="4" t="n">
-        <v>41.75</v>
+        <v>42.75</v>
       </c>
       <c r="B173" s="5" t="n"/>
       <c r="C173" s="6" t="n"/>
@@ -2704,7 +2704,7 @@
     </row>
     <row r="174" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A174" s="4" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B174" s="5" t="n"/>
       <c r="C174" s="6" t="n"/>
@@ -2716,7 +2716,7 @@
     </row>
     <row r="175" hidden="1" outlineLevel="2">
       <c r="A175" s="4" t="n">
-        <v>42.25</v>
+        <v>43.25</v>
       </c>
       <c r="B175" s="5" t="n"/>
       <c r="C175" s="6" t="n"/>
@@ -2728,7 +2728,7 @@
     </row>
     <row r="176" hidden="1" outlineLevel="2">
       <c r="A176" s="4" t="n">
-        <v>42.5</v>
+        <v>43.5</v>
       </c>
       <c r="B176" s="5" t="n"/>
       <c r="C176" s="6" t="n"/>
@@ -2740,7 +2740,7 @@
     </row>
     <row r="177" hidden="1" outlineLevel="2">
       <c r="A177" s="4" t="n">
-        <v>42.75</v>
+        <v>43.75</v>
       </c>
       <c r="B177" s="5" t="n"/>
       <c r="C177" s="6" t="n"/>
@@ -2752,7 +2752,7 @@
     </row>
     <row r="178" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A178" s="4" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B178" s="5" t="n"/>
       <c r="C178" s="6" t="n"/>
@@ -2764,7 +2764,7 @@
     </row>
     <row r="179" hidden="1" outlineLevel="2">
       <c r="A179" s="4" t="n">
-        <v>43.25</v>
+        <v>44.25</v>
       </c>
       <c r="B179" s="5" t="n"/>
       <c r="C179" s="6" t="n"/>
@@ -2776,7 +2776,7 @@
     </row>
     <row r="180" hidden="1" outlineLevel="2">
       <c r="A180" s="4" t="n">
-        <v>43.5</v>
+        <v>44.5</v>
       </c>
       <c r="B180" s="5" t="n"/>
       <c r="C180" s="6" t="n"/>
@@ -2788,7 +2788,7 @@
     </row>
     <row r="181" hidden="1" outlineLevel="2">
       <c r="A181" s="4" t="n">
-        <v>43.75</v>
+        <v>44.75</v>
       </c>
       <c r="B181" s="5" t="n"/>
       <c r="C181" s="6" t="n"/>
@@ -2800,7 +2800,7 @@
     </row>
     <row r="182" collapsed="1" ht="28.8" customHeight="1">
       <c r="A182" s="4" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B182" s="5" t="inlineStr">
         <is>
@@ -2830,7 +2830,7 @@
     </row>
     <row r="183" hidden="1" outlineLevel="2">
       <c r="A183" s="4" t="n">
-        <v>44.25</v>
+        <v>45.25</v>
       </c>
       <c r="B183" s="5" t="n"/>
       <c r="C183" s="6" t="n"/>
@@ -2842,7 +2842,7 @@
     </row>
     <row r="184" hidden="1" outlineLevel="2">
       <c r="A184" s="4" t="n">
-        <v>44.5</v>
+        <v>45.5</v>
       </c>
       <c r="B184" s="5" t="n"/>
       <c r="C184" s="6" t="n"/>
@@ -2854,7 +2854,7 @@
     </row>
     <row r="185" hidden="1" outlineLevel="2">
       <c r="A185" s="4" t="n">
-        <v>44.75</v>
+        <v>45.75</v>
       </c>
       <c r="B185" s="5" t="n"/>
       <c r="C185" s="6" t="n"/>
@@ -2866,7 +2866,7 @@
     </row>
     <row r="186" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A186" s="4" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B186" s="5" t="n"/>
       <c r="C186" s="6" t="n"/>
@@ -2878,7 +2878,7 @@
     </row>
     <row r="187" hidden="1" outlineLevel="2">
       <c r="A187" s="4" t="n">
-        <v>45.25</v>
+        <v>46.25</v>
       </c>
       <c r="B187" s="5" t="n"/>
       <c r="C187" s="6" t="n"/>
@@ -2890,7 +2890,7 @@
     </row>
     <row r="188" hidden="1" outlineLevel="2">
       <c r="A188" s="4" t="n">
-        <v>45.5</v>
+        <v>46.5</v>
       </c>
       <c r="B188" s="5" t="n"/>
       <c r="C188" s="6" t="n"/>
@@ -2902,7 +2902,7 @@
     </row>
     <row r="189" hidden="1" outlineLevel="2">
       <c r="A189" s="4" t="n">
-        <v>45.75</v>
+        <v>46.75</v>
       </c>
       <c r="B189" s="5" t="n"/>
       <c r="C189" s="6" t="n"/>
@@ -2914,7 +2914,7 @@
     </row>
     <row r="190" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A190" s="4" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B190" s="5" t="n"/>
       <c r="C190" s="6" t="n"/>
@@ -2926,7 +2926,7 @@
     </row>
     <row r="191" hidden="1" outlineLevel="2">
       <c r="A191" s="4" t="n">
-        <v>46.25</v>
+        <v>47.25</v>
       </c>
       <c r="B191" s="5" t="n"/>
       <c r="C191" s="6" t="n"/>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="192" hidden="1" outlineLevel="2">
       <c r="A192" s="4" t="n">
-        <v>46.5</v>
+        <v>47.5</v>
       </c>
       <c r="B192" s="5" t="n"/>
       <c r="C192" s="6" t="n"/>
@@ -2950,7 +2950,7 @@
     </row>
     <row r="193" hidden="1" outlineLevel="2">
       <c r="A193" s="4" t="n">
-        <v>46.75</v>
+        <v>47.75</v>
       </c>
       <c r="B193" s="5" t="n"/>
       <c r="C193" s="6" t="n"/>
@@ -2962,7 +2962,7 @@
     </row>
     <row r="194" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A194" s="4" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B194" s="5" t="n"/>
       <c r="C194" s="6" t="n"/>
@@ -2974,7 +2974,7 @@
     </row>
     <row r="195" hidden="1" outlineLevel="2">
       <c r="A195" s="4" t="n">
-        <v>47.25</v>
+        <v>48.25</v>
       </c>
       <c r="B195" s="5" t="n"/>
       <c r="C195" s="6" t="n"/>
@@ -2986,7 +2986,7 @@
     </row>
     <row r="196" hidden="1" outlineLevel="2">
       <c r="A196" s="4" t="n">
-        <v>47.5</v>
+        <v>48.5</v>
       </c>
       <c r="B196" s="5" t="n"/>
       <c r="C196" s="6" t="n"/>
@@ -2998,7 +2998,7 @@
     </row>
     <row r="197" hidden="1" outlineLevel="2">
       <c r="A197" s="4" t="n">
-        <v>47.75</v>
+        <v>48.75</v>
       </c>
       <c r="B197" s="5" t="n"/>
       <c r="C197" s="6" t="n"/>
@@ -3010,7 +3010,7 @@
     </row>
     <row r="198" collapsed="1" ht="28.8" customHeight="1">
       <c r="A198" s="4" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B198" s="5" t="inlineStr">
         <is>
@@ -3040,7 +3040,7 @@
     </row>
     <row r="199" hidden="1" outlineLevel="2">
       <c r="A199" s="4" t="n">
-        <v>48.25</v>
+        <v>49.25</v>
       </c>
       <c r="B199" s="5" t="n"/>
       <c r="C199" s="6" t="n"/>
@@ -3052,7 +3052,7 @@
     </row>
     <row r="200" hidden="1" outlineLevel="2">
       <c r="A200" s="4" t="n">
-        <v>48.5</v>
+        <v>49.5</v>
       </c>
       <c r="B200" s="5" t="n"/>
       <c r="C200" s="6" t="n"/>
@@ -3064,7 +3064,7 @@
     </row>
     <row r="201" hidden="1" outlineLevel="2">
       <c r="A201" s="4" t="n">
-        <v>48.75</v>
+        <v>49.75</v>
       </c>
       <c r="B201" s="5" t="n"/>
       <c r="C201" s="6" t="n"/>
@@ -3076,7 +3076,7 @@
     </row>
     <row r="202" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A202" s="4" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B202" s="5" t="n"/>
       <c r="C202" s="6" t="n"/>
@@ -3088,7 +3088,7 @@
     </row>
     <row r="203" hidden="1" outlineLevel="2">
       <c r="A203" s="4" t="n">
-        <v>49.25</v>
+        <v>50.25</v>
       </c>
       <c r="B203" s="5" t="n"/>
       <c r="C203" s="6" t="n"/>
@@ -3100,7 +3100,7 @@
     </row>
     <row r="204" hidden="1" outlineLevel="2">
       <c r="A204" s="4" t="n">
-        <v>49.5</v>
+        <v>50.5</v>
       </c>
       <c r="B204" s="5" t="n"/>
       <c r="C204" s="6" t="n"/>
@@ -3112,7 +3112,7 @@
     </row>
     <row r="205" hidden="1" outlineLevel="2">
       <c r="A205" s="4" t="n">
-        <v>49.75</v>
+        <v>50.75</v>
       </c>
       <c r="B205" s="5" t="n"/>
       <c r="C205" s="6" t="n"/>
@@ -3124,7 +3124,7 @@
     </row>
     <row r="206" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A206" s="4" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B206" s="5" t="n"/>
       <c r="C206" s="6" t="n"/>
@@ -3136,7 +3136,7 @@
     </row>
     <row r="207" hidden="1" outlineLevel="2">
       <c r="A207" s="4" t="n">
-        <v>50.25</v>
+        <v>51.25</v>
       </c>
       <c r="B207" s="5" t="n"/>
       <c r="C207" s="6" t="n"/>
@@ -3148,7 +3148,7 @@
     </row>
     <row r="208" hidden="1" outlineLevel="2">
       <c r="A208" s="4" t="n">
-        <v>50.5</v>
+        <v>51.5</v>
       </c>
       <c r="B208" s="5" t="n"/>
       <c r="C208" s="6" t="n"/>
@@ -3160,7 +3160,7 @@
     </row>
     <row r="209" hidden="1" outlineLevel="2">
       <c r="A209" s="4" t="n">
-        <v>50.75</v>
+        <v>51.75</v>
       </c>
       <c r="B209" s="5" t="n"/>
       <c r="C209" s="6" t="n"/>
@@ -3172,7 +3172,7 @@
     </row>
     <row r="210" collapsed="1" ht="57.6" customHeight="1">
       <c r="A210" s="4" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B210" s="5" t="inlineStr">
         <is>
@@ -3203,7 +3203,7 @@
     </row>
     <row r="211" hidden="1" outlineLevel="2">
       <c r="A211" s="4" t="n">
-        <v>51.25</v>
+        <v>52.25</v>
       </c>
       <c r="B211" s="5" t="n"/>
       <c r="C211" s="6" t="n"/>
@@ -3215,7 +3215,7 @@
     </row>
     <row r="212" hidden="1" outlineLevel="2">
       <c r="A212" s="4" t="n">
-        <v>51.5</v>
+        <v>52.5</v>
       </c>
       <c r="B212" s="5" t="n"/>
       <c r="C212" s="6" t="n"/>
@@ -3227,7 +3227,7 @@
     </row>
     <row r="213" hidden="1" outlineLevel="2">
       <c r="A213" s="4" t="n">
-        <v>51.75</v>
+        <v>52.75</v>
       </c>
       <c r="B213" s="5" t="n"/>
       <c r="C213" s="6" t="n"/>
@@ -3239,7 +3239,7 @@
     </row>
     <row r="214" collapsed="1" ht="72" customHeight="1">
       <c r="A214" s="4" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B214" s="5" t="inlineStr">
         <is>
@@ -3270,7 +3270,7 @@
     </row>
     <row r="215" hidden="1" outlineLevel="2">
       <c r="A215" s="4" t="n">
-        <v>52.25</v>
+        <v>53.25</v>
       </c>
       <c r="B215" s="5" t="n"/>
       <c r="C215" s="6" t="n"/>
@@ -3282,7 +3282,7 @@
     </row>
     <row r="216" hidden="1" outlineLevel="2">
       <c r="A216" s="4" t="n">
-        <v>52.5</v>
+        <v>53.5</v>
       </c>
       <c r="B216" s="5" t="n"/>
       <c r="C216" s="6" t="n"/>
@@ -3294,7 +3294,7 @@
     </row>
     <row r="217" hidden="1" outlineLevel="2">
       <c r="A217" s="4" t="n">
-        <v>52.75</v>
+        <v>53.75</v>
       </c>
       <c r="B217" s="5" t="n"/>
       <c r="C217" s="6" t="n"/>
@@ -3306,7 +3306,7 @@
     </row>
     <row r="218" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A218" s="4" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B218" s="5" t="n"/>
       <c r="C218" s="6" t="n"/>
@@ -3318,7 +3318,7 @@
     </row>
     <row r="219" hidden="1" outlineLevel="2">
       <c r="A219" s="4" t="n">
-        <v>53.25</v>
+        <v>54.25</v>
       </c>
       <c r="B219" s="5" t="n"/>
       <c r="C219" s="6" t="n"/>
@@ -3330,7 +3330,7 @@
     </row>
     <row r="220" hidden="1" outlineLevel="2">
       <c r="A220" s="4" t="n">
-        <v>53.5</v>
+        <v>54.5</v>
       </c>
       <c r="B220" s="5" t="n"/>
       <c r="C220" s="6" t="n"/>
@@ -3342,7 +3342,7 @@
     </row>
     <row r="221" hidden="1" outlineLevel="2">
       <c r="A221" s="4" t="n">
-        <v>53.75</v>
+        <v>54.75</v>
       </c>
       <c r="B221" s="5" t="n"/>
       <c r="C221" s="6" t="n"/>
@@ -3354,7 +3354,7 @@
     </row>
     <row r="222" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A222" s="4" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B222" s="5" t="n"/>
       <c r="C222" s="6" t="n"/>
@@ -3366,7 +3366,7 @@
     </row>
     <row r="223" hidden="1" outlineLevel="2">
       <c r="A223" s="4" t="n">
-        <v>54.25</v>
+        <v>55.25</v>
       </c>
       <c r="B223" s="5" t="n"/>
       <c r="C223" s="6" t="n"/>
@@ -3378,7 +3378,7 @@
     </row>
     <row r="224" hidden="1" outlineLevel="2">
       <c r="A224" s="4" t="n">
-        <v>54.5</v>
+        <v>55.5</v>
       </c>
       <c r="B224" s="5" t="n"/>
       <c r="C224" s="6" t="n"/>
@@ -3390,7 +3390,7 @@
     </row>
     <row r="225" hidden="1" outlineLevel="2">
       <c r="A225" s="4" t="n">
-        <v>54.75</v>
+        <v>55.75</v>
       </c>
       <c r="B225" s="5" t="n"/>
       <c r="C225" s="6" t="n"/>
@@ -3402,7 +3402,7 @@
     </row>
     <row r="226" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A226" s="4" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B226" s="5" t="n"/>
       <c r="C226" s="6" t="n"/>
@@ -3414,7 +3414,7 @@
     </row>
     <row r="227" hidden="1" outlineLevel="2">
       <c r="A227" s="4" t="n">
-        <v>55.25</v>
+        <v>56.25</v>
       </c>
       <c r="B227" s="5" t="n"/>
       <c r="C227" s="6" t="n"/>
@@ -3426,7 +3426,7 @@
     </row>
     <row r="228" hidden="1" outlineLevel="2">
       <c r="A228" s="4" t="n">
-        <v>55.5</v>
+        <v>56.5</v>
       </c>
       <c r="B228" s="5" t="n"/>
       <c r="C228" s="6" t="n"/>
@@ -3438,7 +3438,7 @@
     </row>
     <row r="229" hidden="1" outlineLevel="2">
       <c r="A229" s="4" t="n">
-        <v>55.75</v>
+        <v>56.75</v>
       </c>
       <c r="B229" s="5" t="n"/>
       <c r="C229" s="6" t="n"/>
@@ -3450,7 +3450,7 @@
     </row>
     <row r="230" collapsed="1" ht="100.8" customHeight="1">
       <c r="A230" s="4" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B230" s="5" t="inlineStr">
         <is>
@@ -3482,7 +3482,7 @@
     </row>
     <row r="231" hidden="1" outlineLevel="2">
       <c r="A231" s="4" t="n">
-        <v>56.25</v>
+        <v>57.25</v>
       </c>
       <c r="B231" s="5" t="n"/>
       <c r="C231" s="6" t="n"/>
@@ -3494,7 +3494,7 @@
     </row>
     <row r="232" hidden="1" outlineLevel="2">
       <c r="A232" s="4" t="n">
-        <v>56.5</v>
+        <v>57.5</v>
       </c>
       <c r="B232" s="5" t="n"/>
       <c r="C232" s="6" t="n"/>
@@ -3506,7 +3506,7 @@
     </row>
     <row r="233" hidden="1" outlineLevel="2">
       <c r="A233" s="4" t="n">
-        <v>56.75</v>
+        <v>57.75</v>
       </c>
       <c r="B233" s="5" t="n"/>
       <c r="C233" s="6" t="n"/>
@@ -3518,7 +3518,7 @@
     </row>
     <row r="234" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A234" s="4" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B234" s="5" t="n"/>
       <c r="C234" s="6" t="n"/>
@@ -3530,7 +3530,7 @@
     </row>
     <row r="235" hidden="1" outlineLevel="2">
       <c r="A235" s="4" t="n">
-        <v>57.25</v>
+        <v>58.25</v>
       </c>
       <c r="B235" s="5" t="n"/>
       <c r="C235" s="6" t="n"/>
@@ -3542,7 +3542,7 @@
     </row>
     <row r="236" hidden="1" outlineLevel="2">
       <c r="A236" s="4" t="n">
-        <v>57.5</v>
+        <v>58.5</v>
       </c>
       <c r="B236" s="5" t="n"/>
       <c r="C236" s="6" t="n"/>
@@ -3554,7 +3554,7 @@
     </row>
     <row r="237" hidden="1" outlineLevel="2">
       <c r="A237" s="4" t="n">
-        <v>57.75</v>
+        <v>58.75</v>
       </c>
       <c r="B237" s="5" t="n"/>
       <c r="C237" s="6" t="n"/>
@@ -3566,7 +3566,7 @@
     </row>
     <row r="238" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A238" s="4" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B238" s="5" t="n"/>
       <c r="C238" s="6" t="n"/>
@@ -3578,7 +3578,7 @@
     </row>
     <row r="239" hidden="1" outlineLevel="2">
       <c r="A239" s="4" t="n">
-        <v>58.25</v>
+        <v>59.25</v>
       </c>
       <c r="B239" s="5" t="n"/>
       <c r="C239" s="6" t="n"/>
@@ -3590,7 +3590,7 @@
     </row>
     <row r="240" hidden="1" outlineLevel="2">
       <c r="A240" s="4" t="n">
-        <v>58.5</v>
+        <v>59.5</v>
       </c>
       <c r="B240" s="5" t="n"/>
       <c r="C240" s="6" t="n"/>
@@ -3602,7 +3602,7 @@
     </row>
     <row r="241" hidden="1" outlineLevel="2">
       <c r="A241" s="4" t="n">
-        <v>58.75</v>
+        <v>59.75</v>
       </c>
       <c r="B241" s="5" t="n"/>
       <c r="C241" s="6" t="n"/>
@@ -3614,7 +3614,7 @@
     </row>
     <row r="242" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A242" s="4" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B242" s="5" t="n"/>
       <c r="C242" s="6" t="n"/>
@@ -3626,7 +3626,7 @@
     </row>
     <row r="243" hidden="1" outlineLevel="2">
       <c r="A243" s="4" t="n">
-        <v>59.25</v>
+        <v>60.25</v>
       </c>
       <c r="B243" s="5" t="n"/>
       <c r="C243" s="6" t="n"/>
@@ -3638,7 +3638,7 @@
     </row>
     <row r="244" hidden="1" outlineLevel="2">
       <c r="A244" s="4" t="n">
-        <v>59.5</v>
+        <v>60.5</v>
       </c>
       <c r="B244" s="5" t="n"/>
       <c r="C244" s="6" t="n"/>
@@ -3650,7 +3650,7 @@
     </row>
     <row r="245" hidden="1" outlineLevel="2">
       <c r="A245" s="4" t="n">
-        <v>59.75</v>
+        <v>60.75</v>
       </c>
       <c r="B245" s="5" t="n"/>
       <c r="C245" s="6" t="n"/>
@@ -3662,7 +3662,7 @@
     </row>
     <row r="246" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A246" s="4" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B246" s="5" t="n"/>
       <c r="C246" s="6" t="n"/>
@@ -3674,7 +3674,7 @@
     </row>
     <row r="247" hidden="1" outlineLevel="2">
       <c r="A247" s="4" t="n">
-        <v>60.25</v>
+        <v>61.25</v>
       </c>
       <c r="B247" s="5" t="n"/>
       <c r="C247" s="6" t="n"/>
@@ -3686,7 +3686,7 @@
     </row>
     <row r="248" hidden="1" outlineLevel="2">
       <c r="A248" s="4" t="n">
-        <v>60.5</v>
+        <v>61.5</v>
       </c>
       <c r="B248" s="5" t="n"/>
       <c r="C248" s="6" t="n"/>
@@ -3698,7 +3698,7 @@
     </row>
     <row r="249" hidden="1" outlineLevel="2">
       <c r="A249" s="4" t="n">
-        <v>60.75</v>
+        <v>61.75</v>
       </c>
       <c r="B249" s="5" t="n"/>
       <c r="C249" s="6" t="n"/>
@@ -3710,7 +3710,7 @@
     </row>
     <row r="250" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A250" s="4" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B250" s="5" t="n"/>
       <c r="C250" s="6" t="n"/>
@@ -3722,7 +3722,7 @@
     </row>
     <row r="251" hidden="1" outlineLevel="2">
       <c r="A251" s="4" t="n">
-        <v>61.25</v>
+        <v>62.25</v>
       </c>
       <c r="B251" s="5" t="n"/>
       <c r="C251" s="6" t="n"/>
@@ -3734,7 +3734,7 @@
     </row>
     <row r="252" hidden="1" outlineLevel="2">
       <c r="A252" s="4" t="n">
-        <v>61.5</v>
+        <v>62.5</v>
       </c>
       <c r="B252" s="5" t="n"/>
       <c r="C252" s="6" t="n"/>
@@ -3746,7 +3746,7 @@
     </row>
     <row r="253" hidden="1" outlineLevel="2">
       <c r="A253" s="4" t="n">
-        <v>61.75</v>
+        <v>62.75</v>
       </c>
       <c r="B253" s="5" t="n"/>
       <c r="C253" s="6" t="n"/>
@@ -3758,7 +3758,7 @@
     </row>
     <row r="254" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A254" s="4" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B254" s="5" t="n"/>
       <c r="C254" s="6" t="n"/>
@@ -3770,7 +3770,7 @@
     </row>
     <row r="255" hidden="1" outlineLevel="2">
       <c r="A255" s="4" t="n">
-        <v>62.25</v>
+        <v>63.25</v>
       </c>
       <c r="B255" s="5" t="n"/>
       <c r="C255" s="6" t="n"/>
@@ -3782,7 +3782,7 @@
     </row>
     <row r="256" hidden="1" outlineLevel="2">
       <c r="A256" s="4" t="n">
-        <v>62.5</v>
+        <v>63.5</v>
       </c>
       <c r="B256" s="5" t="n"/>
       <c r="C256" s="6" t="n"/>
@@ -3794,7 +3794,7 @@
     </row>
     <row r="257" hidden="1" outlineLevel="2">
       <c r="A257" s="4" t="n">
-        <v>62.75</v>
+        <v>63.75</v>
       </c>
       <c r="B257" s="5" t="n"/>
       <c r="C257" s="6" t="n"/>
@@ -3806,7 +3806,7 @@
     </row>
     <row r="258" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A258" s="4" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B258" s="5" t="n"/>
       <c r="C258" s="6" t="n"/>
@@ -3818,7 +3818,7 @@
     </row>
     <row r="259" hidden="1" outlineLevel="2">
       <c r="A259" s="4" t="n">
-        <v>63.25</v>
+        <v>64.25</v>
       </c>
       <c r="B259" s="5" t="n"/>
       <c r="C259" s="6" t="n"/>
@@ -3830,7 +3830,7 @@
     </row>
     <row r="260" hidden="1" outlineLevel="2">
       <c r="A260" s="4" t="n">
-        <v>63.5</v>
+        <v>64.5</v>
       </c>
       <c r="B260" s="5" t="n"/>
       <c r="C260" s="6" t="n"/>
@@ -3842,7 +3842,7 @@
     </row>
     <row r="261" hidden="1" outlineLevel="2">
       <c r="A261" s="4" t="n">
-        <v>63.75</v>
+        <v>64.75</v>
       </c>
       <c r="B261" s="5" t="n"/>
       <c r="C261" s="6" t="n"/>
@@ -3854,7 +3854,7 @@
     </row>
     <row r="262" collapsed="1" ht="86.40000000000001" customHeight="1">
       <c r="A262" s="4" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B262" s="5" t="inlineStr">
         <is>
@@ -3886,7 +3886,7 @@
     </row>
     <row r="263" hidden="1" outlineLevel="2">
       <c r="A263" s="4" t="n">
-        <v>64.25</v>
+        <v>65.25</v>
       </c>
       <c r="B263" s="5" t="n"/>
       <c r="C263" s="6" t="n"/>
@@ -3898,7 +3898,7 @@
     </row>
     <row r="264" hidden="1" outlineLevel="2">
       <c r="A264" s="4" t="n">
-        <v>64.5</v>
+        <v>65.5</v>
       </c>
       <c r="B264" s="5" t="n"/>
       <c r="C264" s="6" t="n"/>
@@ -3910,7 +3910,7 @@
     </row>
     <row r="265" hidden="1" outlineLevel="2">
       <c r="A265" s="4" t="n">
-        <v>64.75</v>
+        <v>65.75</v>
       </c>
       <c r="B265" s="5" t="n"/>
       <c r="C265" s="6" t="n"/>
@@ -3922,7 +3922,7 @@
     </row>
     <row r="266" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A266" s="4" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B266" s="5" t="n"/>
       <c r="C266" s="6" t="n"/>
@@ -3934,7 +3934,7 @@
     </row>
     <row r="267" hidden="1" outlineLevel="2">
       <c r="A267" s="4" t="n">
-        <v>65.25</v>
+        <v>66.25</v>
       </c>
       <c r="B267" s="5" t="n"/>
       <c r="C267" s="6" t="n"/>
@@ -3946,7 +3946,7 @@
     </row>
     <row r="268" hidden="1" outlineLevel="2">
       <c r="A268" s="4" t="n">
-        <v>65.5</v>
+        <v>66.5</v>
       </c>
       <c r="B268" s="5" t="n"/>
       <c r="C268" s="6" t="n"/>
@@ -3958,7 +3958,7 @@
     </row>
     <row r="269" hidden="1" outlineLevel="2">
       <c r="A269" s="4" t="n">
-        <v>65.75</v>
+        <v>66.75</v>
       </c>
       <c r="B269" s="5" t="n"/>
       <c r="C269" s="6" t="n"/>
@@ -3970,7 +3970,7 @@
     </row>
     <row r="270" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A270" s="4" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B270" s="5" t="n"/>
       <c r="C270" s="6" t="n"/>
@@ -3982,7 +3982,7 @@
     </row>
     <row r="271" hidden="1" outlineLevel="2">
       <c r="A271" s="4" t="n">
-        <v>66.25</v>
+        <v>67.25</v>
       </c>
       <c r="B271" s="5" t="n"/>
       <c r="C271" s="6" t="n"/>
@@ -3994,7 +3994,7 @@
     </row>
     <row r="272" hidden="1" outlineLevel="2">
       <c r="A272" s="4" t="n">
-        <v>66.5</v>
+        <v>67.5</v>
       </c>
       <c r="B272" s="5" t="n"/>
       <c r="C272" s="6" t="n"/>
@@ -4006,7 +4006,7 @@
     </row>
     <row r="273" hidden="1" outlineLevel="2">
       <c r="A273" s="4" t="n">
-        <v>66.75</v>
+        <v>67.75</v>
       </c>
       <c r="B273" s="5" t="n"/>
       <c r="C273" s="6" t="n"/>
@@ -4018,7 +4018,7 @@
     </row>
     <row r="274" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A274" s="4" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B274" s="5" t="n"/>
       <c r="C274" s="6" t="n"/>
@@ -4030,7 +4030,7 @@
     </row>
     <row r="275" hidden="1" outlineLevel="2">
       <c r="A275" s="4" t="n">
-        <v>67.25</v>
+        <v>68.25</v>
       </c>
       <c r="B275" s="5" t="n"/>
       <c r="C275" s="6" t="n"/>
@@ -4042,7 +4042,7 @@
     </row>
     <row r="276" hidden="1" outlineLevel="2">
       <c r="A276" s="4" t="n">
-        <v>67.5</v>
+        <v>68.5</v>
       </c>
       <c r="B276" s="5" t="n"/>
       <c r="C276" s="6" t="n"/>
@@ -4054,7 +4054,7 @@
     </row>
     <row r="277" hidden="1" outlineLevel="2">
       <c r="A277" s="4" t="n">
-        <v>67.75</v>
+        <v>68.75</v>
       </c>
       <c r="B277" s="5" t="n"/>
       <c r="C277" s="6" t="n"/>
@@ -4066,7 +4066,7 @@
     </row>
     <row r="278" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A278" s="4" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B278" s="5" t="n"/>
       <c r="C278" s="6" t="n"/>
@@ -4078,7 +4078,7 @@
     </row>
     <row r="279" hidden="1" outlineLevel="2">
       <c r="A279" s="4" t="n">
-        <v>68.25</v>
+        <v>69.25</v>
       </c>
       <c r="B279" s="5" t="n"/>
       <c r="C279" s="6" t="n"/>
@@ -4090,7 +4090,7 @@
     </row>
     <row r="280" hidden="1" outlineLevel="2">
       <c r="A280" s="4" t="n">
-        <v>68.5</v>
+        <v>69.5</v>
       </c>
       <c r="B280" s="5" t="n"/>
       <c r="C280" s="6" t="n"/>
@@ -4102,7 +4102,7 @@
     </row>
     <row r="281" hidden="1" outlineLevel="2">
       <c r="A281" s="4" t="n">
-        <v>68.75</v>
+        <v>69.75</v>
       </c>
       <c r="B281" s="5" t="n"/>
       <c r="C281" s="6" t="n"/>
@@ -4114,7 +4114,7 @@
     </row>
     <row r="282" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A282" s="4" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B282" s="5" t="n"/>
       <c r="C282" s="6" t="n"/>
@@ -4126,7 +4126,7 @@
     </row>
     <row r="283" hidden="1" outlineLevel="2">
       <c r="A283" s="4" t="n">
-        <v>69.25</v>
+        <v>70.25</v>
       </c>
       <c r="B283" s="5" t="n"/>
       <c r="C283" s="6" t="n"/>
@@ -4138,7 +4138,7 @@
     </row>
     <row r="284" hidden="1" outlineLevel="2">
       <c r="A284" s="4" t="n">
-        <v>69.5</v>
+        <v>70.5</v>
       </c>
       <c r="B284" s="5" t="n"/>
       <c r="C284" s="6" t="n"/>
@@ -4150,7 +4150,7 @@
     </row>
     <row r="285" hidden="1" outlineLevel="2">
       <c r="A285" s="4" t="n">
-        <v>69.75</v>
+        <v>70.75</v>
       </c>
       <c r="B285" s="5" t="n"/>
       <c r="C285" s="6" t="n"/>
@@ -4162,7 +4162,7 @@
     </row>
     <row r="286" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A286" s="4" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B286" s="5" t="n"/>
       <c r="C286" s="6" t="n"/>
@@ -4174,7 +4174,7 @@
     </row>
     <row r="287" hidden="1" outlineLevel="2">
       <c r="A287" s="4" t="n">
-        <v>70.25</v>
+        <v>71.25</v>
       </c>
       <c r="B287" s="5" t="n"/>
       <c r="C287" s="6" t="n"/>
@@ -4186,7 +4186,7 @@
     </row>
     <row r="288" hidden="1" outlineLevel="2">
       <c r="A288" s="4" t="n">
-        <v>70.5</v>
+        <v>71.5</v>
       </c>
       <c r="B288" s="5" t="n"/>
       <c r="C288" s="6" t="n"/>
@@ -4198,7 +4198,7 @@
     </row>
     <row r="289" hidden="1" outlineLevel="2">
       <c r="A289" s="4" t="n">
-        <v>70.75</v>
+        <v>71.75</v>
       </c>
       <c r="B289" s="5" t="n"/>
       <c r="C289" s="6" t="n"/>
@@ -4210,7 +4210,7 @@
     </row>
     <row r="290" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A290" s="4" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B290" s="5" t="n"/>
       <c r="C290" s="6" t="n"/>
@@ -4222,7 +4222,7 @@
     </row>
     <row r="291" hidden="1" outlineLevel="2">
       <c r="A291" s="4" t="n">
-        <v>71.25</v>
+        <v>72.25</v>
       </c>
       <c r="B291" s="5" t="n"/>
       <c r="C291" s="6" t="n"/>
@@ -4234,7 +4234,7 @@
     </row>
     <row r="292" hidden="1" outlineLevel="2">
       <c r="A292" s="4" t="n">
-        <v>71.5</v>
+        <v>72.5</v>
       </c>
       <c r="B292" s="5" t="n"/>
       <c r="C292" s="6" t="n"/>
@@ -4246,7 +4246,7 @@
     </row>
     <row r="293" hidden="1" outlineLevel="2">
       <c r="A293" s="4" t="n">
-        <v>71.75</v>
+        <v>72.75</v>
       </c>
       <c r="B293" s="5" t="n"/>
       <c r="C293" s="6" t="n"/>
@@ -4258,7 +4258,7 @@
     </row>
     <row r="294" collapsed="1" ht="100.8" customHeight="1">
       <c r="A294" s="4" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B294" s="5" t="inlineStr">
         <is>
@@ -4290,7 +4290,7 @@
     </row>
     <row r="295" hidden="1" outlineLevel="2">
       <c r="A295" s="4" t="n">
-        <v>72.25</v>
+        <v>73.25</v>
       </c>
       <c r="B295" s="5" t="n"/>
       <c r="C295" s="6" t="n"/>
@@ -4302,7 +4302,7 @@
     </row>
     <row r="296" hidden="1" outlineLevel="2">
       <c r="A296" s="4" t="n">
-        <v>72.5</v>
+        <v>73.5</v>
       </c>
       <c r="B296" s="5" t="n"/>
       <c r="C296" s="6" t="n"/>
@@ -4314,7 +4314,7 @@
     </row>
     <row r="297" hidden="1" outlineLevel="2">
       <c r="A297" s="4" t="n">
-        <v>72.75</v>
+        <v>73.75</v>
       </c>
       <c r="B297" s="5" t="n"/>
       <c r="C297" s="6" t="n"/>
@@ -4326,7 +4326,7 @@
     </row>
     <row r="298" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A298" s="4" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B298" s="5" t="n"/>
       <c r="C298" s="6" t="n"/>
@@ -4338,7 +4338,7 @@
     </row>
     <row r="299" hidden="1" outlineLevel="2">
       <c r="A299" s="4" t="n">
-        <v>73.25</v>
+        <v>74.25</v>
       </c>
       <c r="B299" s="5" t="n"/>
       <c r="C299" s="6" t="n"/>
@@ -4350,7 +4350,7 @@
     </row>
     <row r="300" hidden="1" outlineLevel="2">
       <c r="A300" s="4" t="n">
-        <v>73.5</v>
+        <v>74.5</v>
       </c>
       <c r="B300" s="5" t="n"/>
       <c r="C300" s="6" t="n"/>
@@ -4362,7 +4362,7 @@
     </row>
     <row r="301" hidden="1" outlineLevel="2">
       <c r="A301" s="4" t="n">
-        <v>73.75</v>
+        <v>74.75</v>
       </c>
       <c r="B301" s="5" t="n"/>
       <c r="C301" s="6" t="n"/>
@@ -4374,7 +4374,7 @@
     </row>
     <row r="302" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A302" s="4" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B302" s="5" t="n"/>
       <c r="C302" s="6" t="n"/>
@@ -4386,7 +4386,7 @@
     </row>
     <row r="303" hidden="1" outlineLevel="2">
       <c r="A303" s="4" t="n">
-        <v>74.25</v>
+        <v>75.25</v>
       </c>
       <c r="B303" s="5" t="n"/>
       <c r="C303" s="6" t="n"/>
@@ -4398,7 +4398,7 @@
     </row>
     <row r="304" hidden="1" outlineLevel="2">
       <c r="A304" s="4" t="n">
-        <v>74.5</v>
+        <v>75.5</v>
       </c>
       <c r="B304" s="5" t="n"/>
       <c r="C304" s="6" t="n"/>
@@ -4410,7 +4410,7 @@
     </row>
     <row r="305" hidden="1" outlineLevel="2">
       <c r="A305" s="4" t="n">
-        <v>74.75</v>
+        <v>75.75</v>
       </c>
       <c r="B305" s="5" t="n"/>
       <c r="C305" s="6" t="n"/>
@@ -4422,7 +4422,7 @@
     </row>
     <row r="306" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A306" s="4" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B306" s="5" t="n"/>
       <c r="C306" s="6" t="n"/>
@@ -4434,7 +4434,7 @@
     </row>
     <row r="307" hidden="1" outlineLevel="2">
       <c r="A307" s="4" t="n">
-        <v>75.25</v>
+        <v>76.25</v>
       </c>
       <c r="B307" s="5" t="n"/>
       <c r="C307" s="6" t="n"/>
@@ -4446,7 +4446,7 @@
     </row>
     <row r="308" hidden="1" outlineLevel="2">
       <c r="A308" s="4" t="n">
-        <v>75.5</v>
+        <v>76.5</v>
       </c>
       <c r="B308" s="5" t="n"/>
       <c r="C308" s="6" t="n"/>
@@ -4458,7 +4458,7 @@
     </row>
     <row r="309" hidden="1" outlineLevel="2">
       <c r="A309" s="4" t="n">
-        <v>75.75</v>
+        <v>76.75</v>
       </c>
       <c r="B309" s="5" t="n"/>
       <c r="C309" s="6" t="n"/>
@@ -4470,7 +4470,7 @@
     </row>
     <row r="310" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A310" s="4" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B310" s="5" t="n"/>
       <c r="C310" s="6" t="n"/>
@@ -4482,7 +4482,7 @@
     </row>
     <row r="311" hidden="1" outlineLevel="2">
       <c r="A311" s="4" t="n">
-        <v>76.25</v>
+        <v>77.25</v>
       </c>
       <c r="B311" s="5" t="n"/>
       <c r="C311" s="6" t="n"/>
@@ -4494,7 +4494,7 @@
     </row>
     <row r="312" hidden="1" outlineLevel="2">
       <c r="A312" s="4" t="n">
-        <v>76.5</v>
+        <v>77.5</v>
       </c>
       <c r="B312" s="5" t="n"/>
       <c r="C312" s="6" t="n"/>
@@ -4506,7 +4506,7 @@
     </row>
     <row r="313" hidden="1" outlineLevel="2">
       <c r="A313" s="4" t="n">
-        <v>76.75</v>
+        <v>77.75</v>
       </c>
       <c r="B313" s="5" t="n"/>
       <c r="C313" s="6" t="n"/>
@@ -4518,7 +4518,7 @@
     </row>
     <row r="314" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A314" s="4" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B314" s="5" t="n"/>
       <c r="C314" s="6" t="n"/>
@@ -4530,7 +4530,7 @@
     </row>
     <row r="315" hidden="1" outlineLevel="2">
       <c r="A315" s="4" t="n">
-        <v>77.25</v>
+        <v>78.25</v>
       </c>
       <c r="B315" s="5" t="n"/>
       <c r="C315" s="6" t="n"/>
@@ -4542,7 +4542,7 @@
     </row>
     <row r="316" hidden="1" outlineLevel="2">
       <c r="A316" s="4" t="n">
-        <v>77.5</v>
+        <v>78.5</v>
       </c>
       <c r="B316" s="5" t="n"/>
       <c r="C316" s="6" t="n"/>
@@ -4554,7 +4554,7 @@
     </row>
     <row r="317" hidden="1" outlineLevel="2">
       <c r="A317" s="4" t="n">
-        <v>77.75</v>
+        <v>78.75</v>
       </c>
       <c r="B317" s="5" t="n"/>
       <c r="C317" s="6" t="n"/>
@@ -4566,7 +4566,7 @@
     </row>
     <row r="318" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A318" s="4" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B318" s="5" t="n"/>
       <c r="C318" s="6" t="n"/>
@@ -4578,7 +4578,7 @@
     </row>
     <row r="319" hidden="1" outlineLevel="2">
       <c r="A319" s="4" t="n">
-        <v>78.25</v>
+        <v>79.25</v>
       </c>
       <c r="B319" s="5" t="n"/>
       <c r="C319" s="6" t="n"/>
@@ -4590,7 +4590,7 @@
     </row>
     <row r="320" hidden="1" outlineLevel="2">
       <c r="A320" s="4" t="n">
-        <v>78.5</v>
+        <v>79.5</v>
       </c>
       <c r="B320" s="5" t="n"/>
       <c r="C320" s="6" t="n"/>
@@ -4602,7 +4602,7 @@
     </row>
     <row r="321" hidden="1" outlineLevel="2">
       <c r="A321" s="4" t="n">
-        <v>78.75</v>
+        <v>79.75</v>
       </c>
       <c r="B321" s="5" t="n"/>
       <c r="C321" s="6" t="n"/>
@@ -4614,7 +4614,7 @@
     </row>
     <row r="322" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A322" s="4" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B322" s="5" t="n"/>
       <c r="C322" s="6" t="n"/>
@@ -4626,7 +4626,7 @@
     </row>
     <row r="323" hidden="1" outlineLevel="2">
       <c r="A323" s="4" t="n">
-        <v>79.25</v>
+        <v>80.25</v>
       </c>
       <c r="B323" s="5" t="n"/>
       <c r="C323" s="6" t="n"/>
@@ -4638,7 +4638,7 @@
     </row>
     <row r="324" hidden="1" outlineLevel="2">
       <c r="A324" s="4" t="n">
-        <v>79.5</v>
+        <v>80.5</v>
       </c>
       <c r="B324" s="5" t="n"/>
       <c r="C324" s="6" t="n"/>
@@ -4650,7 +4650,7 @@
     </row>
     <row r="325" hidden="1" outlineLevel="2">
       <c r="A325" s="4" t="n">
-        <v>79.75</v>
+        <v>80.75</v>
       </c>
       <c r="B325" s="5" t="n"/>
       <c r="C325" s="6" t="n"/>
@@ -4662,7 +4662,7 @@
     </row>
     <row r="326" collapsed="1" ht="72" customHeight="1">
       <c r="A326" s="4" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B326" s="5" t="inlineStr">
         <is>
@@ -4694,7 +4694,7 @@
     </row>
     <row r="327" hidden="1" outlineLevel="2">
       <c r="A327" s="4" t="n">
-        <v>80.25</v>
+        <v>81.25</v>
       </c>
       <c r="B327" s="5" t="n"/>
       <c r="C327" s="6" t="n"/>
@@ -4706,7 +4706,7 @@
     </row>
     <row r="328" hidden="1" outlineLevel="2">
       <c r="A328" s="4" t="n">
-        <v>80.5</v>
+        <v>81.5</v>
       </c>
       <c r="B328" s="5" t="n"/>
       <c r="C328" s="6" t="n"/>
@@ -4718,7 +4718,7 @@
     </row>
     <row r="329" hidden="1" outlineLevel="2">
       <c r="A329" s="4" t="n">
-        <v>80.75</v>
+        <v>81.75</v>
       </c>
       <c r="B329" s="5" t="n"/>
       <c r="C329" s="6" t="n"/>
@@ -4730,7 +4730,7 @@
     </row>
     <row r="330" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A330" s="4" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B330" s="5" t="n"/>
       <c r="C330" s="6" t="n"/>
@@ -4742,7 +4742,7 @@
     </row>
     <row r="331" hidden="1" outlineLevel="2">
       <c r="A331" s="4" t="n">
-        <v>81.25</v>
+        <v>82.25</v>
       </c>
       <c r="B331" s="5" t="n"/>
       <c r="C331" s="6" t="n"/>
@@ -4754,7 +4754,7 @@
     </row>
     <row r="332" hidden="1" outlineLevel="2">
       <c r="A332" s="4" t="n">
-        <v>81.5</v>
+        <v>82.5</v>
       </c>
       <c r="B332" s="5" t="n"/>
       <c r="C332" s="6" t="n"/>
@@ -4766,7 +4766,7 @@
     </row>
     <row r="333" hidden="1" outlineLevel="2">
       <c r="A333" s="4" t="n">
-        <v>81.75</v>
+        <v>82.75</v>
       </c>
       <c r="B333" s="5" t="n"/>
       <c r="C333" s="6" t="n"/>
@@ -4778,7 +4778,7 @@
     </row>
     <row r="334" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A334" s="4" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B334" s="5" t="n"/>
       <c r="C334" s="6" t="n"/>
@@ -4790,7 +4790,7 @@
     </row>
     <row r="335" hidden="1" outlineLevel="2">
       <c r="A335" s="4" t="n">
-        <v>82.25</v>
+        <v>83.25</v>
       </c>
       <c r="B335" s="5" t="n"/>
       <c r="C335" s="6" t="n"/>
@@ -4802,7 +4802,7 @@
     </row>
     <row r="336" hidden="1" outlineLevel="2">
       <c r="A336" s="4" t="n">
-        <v>82.5</v>
+        <v>83.5</v>
       </c>
       <c r="B336" s="5" t="n"/>
       <c r="C336" s="6" t="n"/>
@@ -4814,7 +4814,7 @@
     </row>
     <row r="337" hidden="1" outlineLevel="2">
       <c r="A337" s="4" t="n">
-        <v>82.75</v>
+        <v>83.75</v>
       </c>
       <c r="B337" s="5" t="n"/>
       <c r="C337" s="6" t="n"/>
@@ -4826,7 +4826,7 @@
     </row>
     <row r="338" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A338" s="4" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B338" s="5" t="n"/>
       <c r="C338" s="6" t="n"/>
@@ -4838,7 +4838,7 @@
     </row>
     <row r="339" hidden="1" outlineLevel="2">
       <c r="A339" s="4" t="n">
-        <v>83.25</v>
+        <v>84.25</v>
       </c>
       <c r="B339" s="5" t="n"/>
       <c r="C339" s="6" t="n"/>
@@ -4850,7 +4850,7 @@
     </row>
     <row r="340" hidden="1" outlineLevel="2">
       <c r="A340" s="4" t="n">
-        <v>83.5</v>
+        <v>84.5</v>
       </c>
       <c r="B340" s="5" t="n"/>
       <c r="C340" s="6" t="n"/>
@@ -4862,7 +4862,7 @@
     </row>
     <row r="341" hidden="1" outlineLevel="2">
       <c r="A341" s="4" t="n">
-        <v>83.75</v>
+        <v>84.75</v>
       </c>
       <c r="B341" s="5" t="n"/>
       <c r="C341" s="6" t="n"/>
@@ -4874,7 +4874,7 @@
     </row>
     <row r="342" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A342" s="4" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B342" s="5" t="n"/>
       <c r="C342" s="6" t="n"/>
@@ -4886,7 +4886,7 @@
     </row>
     <row r="343" hidden="1" outlineLevel="2">
       <c r="A343" s="4" t="n">
-        <v>84.25</v>
+        <v>85.25</v>
       </c>
       <c r="B343" s="5" t="n"/>
       <c r="C343" s="6" t="n"/>
@@ -4898,7 +4898,7 @@
     </row>
     <row r="344" hidden="1" outlineLevel="2">
       <c r="A344" s="4" t="n">
-        <v>84.5</v>
+        <v>85.5</v>
       </c>
       <c r="B344" s="5" t="n"/>
       <c r="C344" s="6" t="n"/>
@@ -4910,7 +4910,7 @@
     </row>
     <row r="345" hidden="1" outlineLevel="2">
       <c r="A345" s="4" t="n">
-        <v>84.75</v>
+        <v>85.75</v>
       </c>
       <c r="B345" s="5" t="n"/>
       <c r="C345" s="6" t="n"/>
@@ -4922,7 +4922,7 @@
     </row>
     <row r="346" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A346" s="4" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B346" s="5" t="n"/>
       <c r="C346" s="6" t="n"/>
@@ -4934,7 +4934,7 @@
     </row>
     <row r="347" hidden="1" outlineLevel="2">
       <c r="A347" s="4" t="n">
-        <v>85.25</v>
+        <v>86.25</v>
       </c>
       <c r="B347" s="5" t="n"/>
       <c r="C347" s="6" t="n"/>
@@ -4946,7 +4946,7 @@
     </row>
     <row r="348" hidden="1" outlineLevel="2">
       <c r="A348" s="4" t="n">
-        <v>85.5</v>
+        <v>86.5</v>
       </c>
       <c r="B348" s="5" t="n"/>
       <c r="C348" s="6" t="n"/>
@@ -4958,7 +4958,7 @@
     </row>
     <row r="349" hidden="1" outlineLevel="2">
       <c r="A349" s="4" t="n">
-        <v>85.75</v>
+        <v>86.75</v>
       </c>
       <c r="B349" s="5" t="n"/>
       <c r="C349" s="6" t="n"/>
@@ -4970,7 +4970,7 @@
     </row>
     <row r="350" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A350" s="4" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B350" s="5" t="n"/>
       <c r="C350" s="6" t="n"/>
@@ -4982,7 +4982,7 @@
     </row>
     <row r="351" hidden="1" outlineLevel="2">
       <c r="A351" s="4" t="n">
-        <v>86.25</v>
+        <v>87.25</v>
       </c>
       <c r="B351" s="5" t="n"/>
       <c r="C351" s="6" t="n"/>
@@ -4994,7 +4994,7 @@
     </row>
     <row r="352" hidden="1" outlineLevel="2">
       <c r="A352" s="4" t="n">
-        <v>86.5</v>
+        <v>87.5</v>
       </c>
       <c r="B352" s="5" t="n"/>
       <c r="C352" s="6" t="n"/>
@@ -5006,7 +5006,7 @@
     </row>
     <row r="353" hidden="1" outlineLevel="2">
       <c r="A353" s="4" t="n">
-        <v>86.75</v>
+        <v>87.75</v>
       </c>
       <c r="B353" s="5" t="n"/>
       <c r="C353" s="6" t="n"/>
@@ -5018,7 +5018,7 @@
     </row>
     <row r="354" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A354" s="4" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B354" s="5" t="n"/>
       <c r="C354" s="6" t="n"/>
@@ -5030,7 +5030,7 @@
     </row>
     <row r="355" hidden="1" outlineLevel="2">
       <c r="A355" s="4" t="n">
-        <v>87.25</v>
+        <v>88.25</v>
       </c>
       <c r="B355" s="5" t="n"/>
       <c r="C355" s="6" t="n"/>
@@ -5042,7 +5042,7 @@
     </row>
     <row r="356" hidden="1" outlineLevel="2">
       <c r="A356" s="4" t="n">
-        <v>87.5</v>
+        <v>88.5</v>
       </c>
       <c r="B356" s="5" t="n"/>
       <c r="C356" s="6" t="n"/>
@@ -5054,7 +5054,7 @@
     </row>
     <row r="357" hidden="1" outlineLevel="2">
       <c r="A357" s="4" t="n">
-        <v>87.75</v>
+        <v>88.75</v>
       </c>
       <c r="B357" s="5" t="n"/>
       <c r="C357" s="6" t="n"/>
@@ -5066,7 +5066,7 @@
     </row>
     <row r="358" collapsed="1" ht="43.2" customHeight="1">
       <c r="A358" s="4" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B358" s="5" t="inlineStr">
         <is>
@@ -5096,7 +5096,7 @@
     </row>
     <row r="359" hidden="1" outlineLevel="2">
       <c r="A359" s="4" t="n">
-        <v>88.25</v>
+        <v>89.25</v>
       </c>
       <c r="B359" s="5" t="n"/>
       <c r="C359" s="6" t="n"/>
@@ -5108,7 +5108,7 @@
     </row>
     <row r="360" hidden="1" outlineLevel="2">
       <c r="A360" s="4" t="n">
-        <v>88.5</v>
+        <v>89.5</v>
       </c>
       <c r="B360" s="5" t="n"/>
       <c r="C360" s="6" t="n"/>
@@ -5120,7 +5120,7 @@
     </row>
     <row r="361" hidden="1" outlineLevel="2">
       <c r="A361" s="4" t="n">
-        <v>88.75</v>
+        <v>89.75</v>
       </c>
       <c r="B361" s="5" t="n"/>
       <c r="C361" s="6" t="n"/>
@@ -5132,7 +5132,7 @@
     </row>
     <row r="362" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A362" s="4" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B362" s="5" t="n"/>
       <c r="C362" s="6" t="n"/>
@@ -5144,7 +5144,7 @@
     </row>
     <row r="363" hidden="1" outlineLevel="2">
       <c r="A363" s="4" t="n">
-        <v>89.25</v>
+        <v>90.25</v>
       </c>
       <c r="B363" s="5" t="n"/>
       <c r="C363" s="6" t="n"/>
@@ -5156,7 +5156,7 @@
     </row>
     <row r="364" hidden="1" outlineLevel="2">
       <c r="A364" s="4" t="n">
-        <v>89.5</v>
+        <v>90.5</v>
       </c>
       <c r="B364" s="5" t="n"/>
       <c r="C364" s="6" t="n"/>
@@ -5168,7 +5168,7 @@
     </row>
     <row r="365" hidden="1" outlineLevel="2">
       <c r="A365" s="4" t="n">
-        <v>89.75</v>
+        <v>90.75</v>
       </c>
       <c r="B365" s="5" t="n"/>
       <c r="C365" s="6" t="n"/>
@@ -5180,7 +5180,7 @@
     </row>
     <row r="366" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A366" s="4" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B366" s="5" t="n"/>
       <c r="C366" s="6" t="n"/>
@@ -5192,7 +5192,7 @@
     </row>
     <row r="367" hidden="1" outlineLevel="2">
       <c r="A367" s="4" t="n">
-        <v>90.25</v>
+        <v>91.25</v>
       </c>
       <c r="B367" s="5" t="n"/>
       <c r="C367" s="6" t="n"/>
@@ -5204,7 +5204,7 @@
     </row>
     <row r="368">
       <c r="A368" s="7" t="n">
-        <v>90.5</v>
+        <v>91.5</v>
       </c>
       <c r="B368" t="inlineStr">
         <is>

</xml_diff>